<commit_message>
editted excel to diya code
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yuhang\Coding\dphil_data_processing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{590DE193-8126-403F-9863-D262EC6EAC85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D225EF48-A857-4187-9DF8-A620B19DE0E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Plate data" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="45">
   <si>
     <t>Red</t>
   </si>
@@ -61,6 +61,105 @@
   </si>
   <si>
     <t>Media</t>
+  </si>
+  <si>
+    <t>N-D-1-R</t>
+  </si>
+  <si>
+    <t>N-O-1-R</t>
+  </si>
+  <si>
+    <t>N-D-1-G</t>
+  </si>
+  <si>
+    <t>N-O-1-G</t>
+  </si>
+  <si>
+    <t>N-D-2-R</t>
+  </si>
+  <si>
+    <t>N-O-2-R</t>
+  </si>
+  <si>
+    <t>N-D-2-G</t>
+  </si>
+  <si>
+    <t>N-O-2-G</t>
+  </si>
+  <si>
+    <t>N-D-3-R</t>
+  </si>
+  <si>
+    <t>N-O-3-R</t>
+  </si>
+  <si>
+    <t>N-D-3-G</t>
+  </si>
+  <si>
+    <t>N-O-3-G</t>
+  </si>
+  <si>
+    <t>K-D-1-R</t>
+  </si>
+  <si>
+    <t>K-O-1-R</t>
+  </si>
+  <si>
+    <t>K-D-1-G</t>
+  </si>
+  <si>
+    <t>K-O-1-G</t>
+  </si>
+  <si>
+    <t>K-D-2-R</t>
+  </si>
+  <si>
+    <t>K-O-2-R</t>
+  </si>
+  <si>
+    <t>K-D-2-G</t>
+  </si>
+  <si>
+    <t>K-O-2-G</t>
+  </si>
+  <si>
+    <t>K-D-3-R</t>
+  </si>
+  <si>
+    <t>K-O-3-R</t>
+  </si>
+  <si>
+    <t>K-D-3-G</t>
+  </si>
+  <si>
+    <t>K-O-3-G</t>
+  </si>
+  <si>
+    <t>BCS-D-R</t>
+  </si>
+  <si>
+    <t>BCS-O-R</t>
+  </si>
+  <si>
+    <t>BCS-D-G</t>
+  </si>
+  <si>
+    <t>BCS-O-G</t>
+  </si>
+  <si>
+    <t>BK-D-R</t>
+  </si>
+  <si>
+    <t>BK-O-R</t>
+  </si>
+  <si>
+    <t>BK-D-G</t>
+  </si>
+  <si>
+    <t>BK-O-G</t>
+  </si>
+  <si>
+    <t>LB</t>
   </si>
 </sst>
 </file>
@@ -447,22 +546,22 @@
         <v>2.8</v>
       </c>
       <c r="H3">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="I3">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="J3">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="K3">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="L3">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="M3">
-        <v>2.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.4">
@@ -488,22 +587,22 @@
         <v>2.8</v>
       </c>
       <c r="H4">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="I4">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="J4">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="K4">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="L4">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="M4">
-        <v>2.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.4">
@@ -529,22 +628,22 @@
         <v>2.8</v>
       </c>
       <c r="H5">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="I5">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="J5">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="K5">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="L5">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="M5">
-        <v>2.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.4">
@@ -570,22 +669,22 @@
         <v>2.8</v>
       </c>
       <c r="H6">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="I6">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="J6">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="K6">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="L6">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="M6">
-        <v>2.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.4">
@@ -611,22 +710,22 @@
         <v>2.8</v>
       </c>
       <c r="H7">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="J7">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="K7">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="L7">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="M7">
-        <v>2.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.4">
@@ -652,22 +751,22 @@
         <v>2.8</v>
       </c>
       <c r="H8">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="I8">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="J8">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="K8">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="L8">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="M8">
-        <v>2.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.4">
@@ -693,13 +792,13 @@
         <v>2.8</v>
       </c>
       <c r="H9">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="I9">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="J9">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="K9">
         <v>0</v>
@@ -734,13 +833,13 @@
         <v>2.8</v>
       </c>
       <c r="H10">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="I10">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="J10">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="K10">
         <v>0</v>
@@ -800,10 +899,10 @@
         <v>1</v>
       </c>
       <c r="B15">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="C15">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="D15">
         <v>0</v>
@@ -815,25 +914,25 @@
         <v>0</v>
       </c>
       <c r="G15">
-        <v>0.27999999999999997</v>
+        <v>0</v>
       </c>
       <c r="H15">
-        <v>1.4</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="I15">
-        <v>0</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="J15">
-        <v>1.4</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="K15">
-        <v>0</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="L15">
-        <v>0</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="M15">
-        <v>1.4</v>
+        <v>0.28000000000000003</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.4">
@@ -841,40 +940,40 @@
         <v>2</v>
       </c>
       <c r="B16">
-        <v>0.27999999999999997</v>
+        <v>0</v>
       </c>
       <c r="C16">
-        <v>0.27999999999999997</v>
+        <v>0</v>
       </c>
       <c r="D16">
-        <v>0.27999999999999997</v>
+        <v>0</v>
       </c>
       <c r="E16">
-        <v>0.27999999999999997</v>
+        <v>0</v>
       </c>
       <c r="F16">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="G16">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="H16">
-        <v>0</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="I16">
-        <v>0.27999999999999997</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="J16">
-        <v>0.27999999999999997</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="K16">
-        <v>1.4</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="L16">
-        <v>0.27999999999999997</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="M16">
-        <v>0.27999999999999997</v>
+        <v>0.28000000000000003</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.4">
@@ -888,34 +987,34 @@
         <v>0</v>
       </c>
       <c r="D17">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="E17">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="F17">
-        <v>0.27999999999999997</v>
+        <v>0</v>
       </c>
       <c r="G17">
         <v>0</v>
       </c>
       <c r="H17">
-        <v>0.27999999999999997</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="I17">
-        <v>1.4</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="J17">
-        <v>0</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="K17">
-        <v>0.27999999999999997</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="L17">
-        <v>1.4</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="M17">
-        <v>0</v>
+        <v>0.28000000000000003</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.4">
@@ -923,40 +1022,40 @@
         <v>4</v>
       </c>
       <c r="B18">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="C18">
-        <v>0.27999999999999997</v>
+        <v>0</v>
       </c>
       <c r="D18">
-        <v>0.27999999999999997</v>
+        <v>0</v>
       </c>
       <c r="E18">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="F18">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="G18">
-        <v>0.27999999999999997</v>
+        <v>0</v>
       </c>
       <c r="H18">
-        <v>1.4</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="I18">
-        <v>0</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="J18">
-        <v>1.4</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="K18">
-        <v>0.27999999999999997</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="L18">
-        <v>0</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="M18">
-        <v>1.4</v>
+        <v>0.28000000000000003</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.4">
@@ -964,16 +1063,16 @@
         <v>5</v>
       </c>
       <c r="B19">
-        <v>0.27999999999999997</v>
+        <v>0</v>
       </c>
       <c r="C19">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="D19">
         <v>0</v>
       </c>
       <c r="E19">
-        <v>0.27999999999999997</v>
+        <v>0</v>
       </c>
       <c r="F19">
         <v>0</v>
@@ -982,22 +1081,22 @@
         <v>0</v>
       </c>
       <c r="H19">
-        <v>0</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="I19">
-        <v>0.27999999999999997</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="J19">
-        <v>0</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="K19">
-        <v>1.4</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="L19">
-        <v>0.27999999999999997</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="M19">
-        <v>0</v>
+        <v>0.28000000000000003</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.4">
@@ -1011,34 +1110,34 @@
         <v>0</v>
       </c>
       <c r="D20">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="E20">
         <v>0</v>
       </c>
       <c r="F20">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="G20">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="H20">
-        <v>0</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="I20">
-        <v>1.4</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="J20">
-        <v>0.27999999999999997</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="K20">
-        <v>0</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="L20">
-        <v>1.4</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="M20">
-        <v>0.27999999999999997</v>
+        <v>0.28000000000000003</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.4">
@@ -1046,40 +1145,40 @@
         <v>7</v>
       </c>
       <c r="B21">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="C21">
-        <v>0.27999999999999997</v>
+        <v>0</v>
       </c>
       <c r="D21">
         <v>0</v>
       </c>
       <c r="E21">
-        <v>0.27999999999999997</v>
+        <v>0</v>
       </c>
       <c r="F21">
-        <v>0.27999999999999997</v>
+        <v>0</v>
       </c>
       <c r="G21">
-        <v>0.27999999999999997</v>
+        <v>0</v>
       </c>
       <c r="H21">
-        <v>0.27999999999999997</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="I21">
-        <v>0.27999999999999997</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="J21">
-        <v>1.4</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="K21">
-        <v>0</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="L21">
-        <v>0</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="M21">
-        <v>0</v>
+        <v>0.28000000000000003</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.4">
@@ -1090,10 +1189,10 @@
         <v>0</v>
       </c>
       <c r="C22">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="D22">
-        <v>0.27999999999999997</v>
+        <v>0</v>
       </c>
       <c r="E22">
         <v>0</v>
@@ -1102,25 +1201,25 @@
         <v>0</v>
       </c>
       <c r="G22">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="H22">
-        <v>1.4</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="I22">
-        <v>0</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="J22">
-        <v>0.27999999999999997</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="K22">
-        <v>0</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="L22">
-        <v>0</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="M22">
-        <v>0</v>
+        <v>0.28000000000000003</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.4">
@@ -1170,41 +1269,329 @@
       <c r="A27" t="s">
         <v>1</v>
       </c>
+      <c r="B27" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" t="s">
+        <v>13</v>
+      </c>
+      <c r="F27" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27" t="s">
+        <v>13</v>
+      </c>
+      <c r="H27" t="s">
+        <v>14</v>
+      </c>
+      <c r="I27" t="s">
+        <v>14</v>
+      </c>
+      <c r="J27" t="s">
+        <v>14</v>
+      </c>
+      <c r="K27" t="s">
+        <v>15</v>
+      </c>
+      <c r="L27" t="s">
+        <v>15</v>
+      </c>
+      <c r="M27" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>2</v>
       </c>
+      <c r="B28" t="s">
+        <v>16</v>
+      </c>
+      <c r="C28" t="s">
+        <v>16</v>
+      </c>
+      <c r="D28" t="s">
+        <v>16</v>
+      </c>
+      <c r="E28" t="s">
+        <v>17</v>
+      </c>
+      <c r="F28" t="s">
+        <v>17</v>
+      </c>
+      <c r="G28" t="s">
+        <v>17</v>
+      </c>
+      <c r="H28" t="s">
+        <v>18</v>
+      </c>
+      <c r="I28" t="s">
+        <v>18</v>
+      </c>
+      <c r="J28" t="s">
+        <v>18</v>
+      </c>
+      <c r="K28" t="s">
+        <v>19</v>
+      </c>
+      <c r="L28" t="s">
+        <v>19</v>
+      </c>
+      <c r="M28" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>3</v>
       </c>
+      <c r="B29" t="s">
+        <v>20</v>
+      </c>
+      <c r="C29" t="s">
+        <v>20</v>
+      </c>
+      <c r="D29" t="s">
+        <v>20</v>
+      </c>
+      <c r="E29" t="s">
+        <v>21</v>
+      </c>
+      <c r="F29" t="s">
+        <v>21</v>
+      </c>
+      <c r="G29" t="s">
+        <v>21</v>
+      </c>
+      <c r="H29" t="s">
+        <v>22</v>
+      </c>
+      <c r="I29" t="s">
+        <v>22</v>
+      </c>
+      <c r="J29" t="s">
+        <v>22</v>
+      </c>
+      <c r="K29" t="s">
+        <v>23</v>
+      </c>
+      <c r="L29" t="s">
+        <v>23</v>
+      </c>
+      <c r="M29" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>4</v>
       </c>
+      <c r="B30" t="s">
+        <v>24</v>
+      </c>
+      <c r="C30" t="s">
+        <v>24</v>
+      </c>
+      <c r="D30" t="s">
+        <v>24</v>
+      </c>
+      <c r="E30" t="s">
+        <v>25</v>
+      </c>
+      <c r="F30" t="s">
+        <v>25</v>
+      </c>
+      <c r="G30" t="s">
+        <v>25</v>
+      </c>
+      <c r="H30" t="s">
+        <v>26</v>
+      </c>
+      <c r="I30" t="s">
+        <v>26</v>
+      </c>
+      <c r="J30" t="s">
+        <v>26</v>
+      </c>
+      <c r="K30" t="s">
+        <v>27</v>
+      </c>
+      <c r="L30" t="s">
+        <v>27</v>
+      </c>
+      <c r="M30" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>5</v>
       </c>
+      <c r="B31" t="s">
+        <v>28</v>
+      </c>
+      <c r="C31" t="s">
+        <v>28</v>
+      </c>
+      <c r="D31" t="s">
+        <v>28</v>
+      </c>
+      <c r="E31" t="s">
+        <v>29</v>
+      </c>
+      <c r="F31" t="s">
+        <v>29</v>
+      </c>
+      <c r="G31" t="s">
+        <v>29</v>
+      </c>
+      <c r="H31" t="s">
+        <v>30</v>
+      </c>
+      <c r="I31" t="s">
+        <v>30</v>
+      </c>
+      <c r="J31" t="s">
+        <v>30</v>
+      </c>
+      <c r="K31" t="s">
+        <v>31</v>
+      </c>
+      <c r="L31" t="s">
+        <v>31</v>
+      </c>
+      <c r="M31" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>6</v>
       </c>
+      <c r="B32" t="s">
+        <v>32</v>
+      </c>
+      <c r="C32" t="s">
+        <v>32</v>
+      </c>
+      <c r="D32" t="s">
+        <v>32</v>
+      </c>
+      <c r="E32" t="s">
+        <v>33</v>
+      </c>
+      <c r="F32" t="s">
+        <v>33</v>
+      </c>
+      <c r="G32" t="s">
+        <v>33</v>
+      </c>
+      <c r="H32" t="s">
+        <v>34</v>
+      </c>
+      <c r="I32" t="s">
+        <v>34</v>
+      </c>
+      <c r="J32" t="s">
+        <v>34</v>
+      </c>
+      <c r="K32" t="s">
+        <v>35</v>
+      </c>
+      <c r="L32" t="s">
+        <v>35</v>
+      </c>
+      <c r="M32" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
         <v>7</v>
       </c>
+      <c r="B33" t="s">
+        <v>36</v>
+      </c>
+      <c r="C33" t="s">
+        <v>36</v>
+      </c>
+      <c r="D33" t="s">
+        <v>36</v>
+      </c>
+      <c r="E33" t="s">
+        <v>37</v>
+      </c>
+      <c r="F33" t="s">
+        <v>37</v>
+      </c>
+      <c r="G33" t="s">
+        <v>37</v>
+      </c>
+      <c r="H33" t="s">
+        <v>38</v>
+      </c>
+      <c r="I33" t="s">
+        <v>38</v>
+      </c>
+      <c r="J33" t="s">
+        <v>38</v>
+      </c>
+      <c r="K33" t="s">
+        <v>39</v>
+      </c>
+      <c r="L33" t="s">
+        <v>39</v>
+      </c>
+      <c r="M33" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
         <v>8</v>
       </c>
+      <c r="B34" t="s">
+        <v>40</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34" t="s">
+        <v>40</v>
+      </c>
+      <c r="E34" t="s">
+        <v>41</v>
+      </c>
+      <c r="F34" t="s">
+        <v>41</v>
+      </c>
+      <c r="G34" t="s">
+        <v>41</v>
+      </c>
+      <c r="H34" t="s">
+        <v>42</v>
+      </c>
+      <c r="I34" t="s">
+        <v>42</v>
+      </c>
+      <c r="J34" t="s">
+        <v>42</v>
+      </c>
+      <c r="K34" t="s">
+        <v>43</v>
+      </c>
+      <c r="L34" t="s">
+        <v>43</v>
+      </c>
+      <c r="M34" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
@@ -1253,40 +1640,328 @@
       <c r="A39" t="s">
         <v>1</v>
       </c>
+      <c r="B39" t="s">
+        <v>44</v>
+      </c>
+      <c r="C39" t="s">
+        <v>44</v>
+      </c>
+      <c r="D39" t="s">
+        <v>44</v>
+      </c>
+      <c r="E39" t="s">
+        <v>44</v>
+      </c>
+      <c r="F39" t="s">
+        <v>44</v>
+      </c>
+      <c r="G39" t="s">
+        <v>44</v>
+      </c>
+      <c r="H39" t="s">
+        <v>44</v>
+      </c>
+      <c r="I39" t="s">
+        <v>44</v>
+      </c>
+      <c r="J39" t="s">
+        <v>44</v>
+      </c>
+      <c r="K39" t="s">
+        <v>44</v>
+      </c>
+      <c r="L39" t="s">
+        <v>44</v>
+      </c>
+      <c r="M39" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
         <v>2</v>
       </c>
+      <c r="B40" t="s">
+        <v>44</v>
+      </c>
+      <c r="C40" t="s">
+        <v>44</v>
+      </c>
+      <c r="D40" t="s">
+        <v>44</v>
+      </c>
+      <c r="E40" t="s">
+        <v>44</v>
+      </c>
+      <c r="F40" t="s">
+        <v>44</v>
+      </c>
+      <c r="G40" t="s">
+        <v>44</v>
+      </c>
+      <c r="H40" t="s">
+        <v>44</v>
+      </c>
+      <c r="I40" t="s">
+        <v>44</v>
+      </c>
+      <c r="J40" t="s">
+        <v>44</v>
+      </c>
+      <c r="K40" t="s">
+        <v>44</v>
+      </c>
+      <c r="L40" t="s">
+        <v>44</v>
+      </c>
+      <c r="M40" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
         <v>3</v>
       </c>
+      <c r="B41" t="s">
+        <v>44</v>
+      </c>
+      <c r="C41" t="s">
+        <v>44</v>
+      </c>
+      <c r="D41" t="s">
+        <v>44</v>
+      </c>
+      <c r="E41" t="s">
+        <v>44</v>
+      </c>
+      <c r="F41" t="s">
+        <v>44</v>
+      </c>
+      <c r="G41" t="s">
+        <v>44</v>
+      </c>
+      <c r="H41" t="s">
+        <v>44</v>
+      </c>
+      <c r="I41" t="s">
+        <v>44</v>
+      </c>
+      <c r="J41" t="s">
+        <v>44</v>
+      </c>
+      <c r="K41" t="s">
+        <v>44</v>
+      </c>
+      <c r="L41" t="s">
+        <v>44</v>
+      </c>
+      <c r="M41" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>4</v>
       </c>
+      <c r="B42" t="s">
+        <v>44</v>
+      </c>
+      <c r="C42" t="s">
+        <v>44</v>
+      </c>
+      <c r="D42" t="s">
+        <v>44</v>
+      </c>
+      <c r="E42" t="s">
+        <v>44</v>
+      </c>
+      <c r="F42" t="s">
+        <v>44</v>
+      </c>
+      <c r="G42" t="s">
+        <v>44</v>
+      </c>
+      <c r="H42" t="s">
+        <v>44</v>
+      </c>
+      <c r="I42" t="s">
+        <v>44</v>
+      </c>
+      <c r="J42" t="s">
+        <v>44</v>
+      </c>
+      <c r="K42" t="s">
+        <v>44</v>
+      </c>
+      <c r="L42" t="s">
+        <v>44</v>
+      </c>
+      <c r="M42" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
         <v>5</v>
       </c>
+      <c r="B43" t="s">
+        <v>44</v>
+      </c>
+      <c r="C43" t="s">
+        <v>44</v>
+      </c>
+      <c r="D43" t="s">
+        <v>44</v>
+      </c>
+      <c r="E43" t="s">
+        <v>44</v>
+      </c>
+      <c r="F43" t="s">
+        <v>44</v>
+      </c>
+      <c r="G43" t="s">
+        <v>44</v>
+      </c>
+      <c r="H43" t="s">
+        <v>44</v>
+      </c>
+      <c r="I43" t="s">
+        <v>44</v>
+      </c>
+      <c r="J43" t="s">
+        <v>44</v>
+      </c>
+      <c r="K43" t="s">
+        <v>44</v>
+      </c>
+      <c r="L43" t="s">
+        <v>44</v>
+      </c>
+      <c r="M43" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>6</v>
       </c>
+      <c r="B44" t="s">
+        <v>44</v>
+      </c>
+      <c r="C44" t="s">
+        <v>44</v>
+      </c>
+      <c r="D44" t="s">
+        <v>44</v>
+      </c>
+      <c r="E44" t="s">
+        <v>44</v>
+      </c>
+      <c r="F44" t="s">
+        <v>44</v>
+      </c>
+      <c r="G44" t="s">
+        <v>44</v>
+      </c>
+      <c r="H44" t="s">
+        <v>44</v>
+      </c>
+      <c r="I44" t="s">
+        <v>44</v>
+      </c>
+      <c r="J44" t="s">
+        <v>44</v>
+      </c>
+      <c r="K44" t="s">
+        <v>44</v>
+      </c>
+      <c r="L44" t="s">
+        <v>44</v>
+      </c>
+      <c r="M44" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
         <v>7</v>
       </c>
+      <c r="B45" t="s">
+        <v>44</v>
+      </c>
+      <c r="C45" t="s">
+        <v>44</v>
+      </c>
+      <c r="D45" t="s">
+        <v>44</v>
+      </c>
+      <c r="E45" t="s">
+        <v>44</v>
+      </c>
+      <c r="F45" t="s">
+        <v>44</v>
+      </c>
+      <c r="G45" t="s">
+        <v>44</v>
+      </c>
+      <c r="H45" t="s">
+        <v>44</v>
+      </c>
+      <c r="I45" t="s">
+        <v>44</v>
+      </c>
+      <c r="J45" t="s">
+        <v>44</v>
+      </c>
+      <c r="K45" t="s">
+        <v>44</v>
+      </c>
+      <c r="L45" t="s">
+        <v>44</v>
+      </c>
+      <c r="M45" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A46" t="s">
         <v>8</v>
+      </c>
+      <c r="B46" t="s">
+        <v>44</v>
+      </c>
+      <c r="C46" t="s">
+        <v>44</v>
+      </c>
+      <c r="D46" t="s">
+        <v>44</v>
+      </c>
+      <c r="E46" t="s">
+        <v>44</v>
+      </c>
+      <c r="F46" t="s">
+        <v>44</v>
+      </c>
+      <c r="G46" t="s">
+        <v>44</v>
+      </c>
+      <c r="H46" t="s">
+        <v>44</v>
+      </c>
+      <c r="I46" t="s">
+        <v>44</v>
+      </c>
+      <c r="J46" t="s">
+        <v>44</v>
+      </c>
+      <c r="K46" t="s">
+        <v>44</v>
+      </c>
+      <c r="L46" t="s">
+        <v>44</v>
+      </c>
+      <c r="M46" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>